<commit_message>
feat: write VM metadata to Proxmox notes from Excel/CSV source
</commit_message>
<xml_diff>
--- a/files/vm_tags.example.xlsx
+++ b/files/vm_tags.example.xlsx
@@ -413,225 +413,516 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A2:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>VMID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>IP Address</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Disk</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Backup</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>100</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>web-prod-01</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>platform</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nginx</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>daily</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>public;tier-web</t>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Internet Facing</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Criticality</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Business Service</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Contact Group</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>BackupRequired</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>SupportVendor</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>web-prod-02</t>
+          <t>BenWin</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>server1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>platform</t>
+          <t>VM</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>nginx</t>
+          <t>10.1.2.200</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>daily</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>public;tier-web</t>
+          <t>Win10</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>8.0 GB</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>200G</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ben.leung@digitaledgedc.com</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>PRO</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Jumphost for recovery</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>HKGA1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>IT DR</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ITInfra</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>200</v>
+        <v>134</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>db-prod-01</t>
+          <t>lhkgautoinv1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>server1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>dba</t>
+          <t>VM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>postgres</t>
+          <t>10.1.2.54</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>hourly</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>tier-data;pci</t>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>4.0 GB</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>100G</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>wai.kwong@digitaledgedc.com</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PRO</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Proxmox Auto Inventory</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>HKGA1</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Infrastructure Automation</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ITOps</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>300</v>
+        <v>117</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>app-uat-01</t>
+          <t>wireguard</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>server3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>app-team</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>billing</t>
-        </is>
-      </c>
+          <t>VM</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>weekly</t>
+          <t>stopped</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>tier-app</t>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4.0 GB</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>50G</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Kelvin.chia@digitaledgedc.com</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PRO</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>WireGuard</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>HKGA1</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Backdoor VPN for Kelvin</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Kelvin</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>400</v>
+        <v>106</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jenkins-01</t>
+          <t>gideon</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>server2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>devops</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>jenkins</t>
-        </is>
-      </c>
+          <t>VM</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>stopped</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>8.0 GB</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>100G</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Can remove</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>136</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dns1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>server2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Container</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>10.1.2.41</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ubuntu</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2.0 GB</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>10G</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>